<commit_message>
Leads: 2026-10-12 00:04 UTC (cycle 165)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-12.xlsx
+++ b/output/leads_2026-10-12.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -563,6 +563,66 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Stat Roofing and Sheet Metal</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>stat-roofing.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://stat-roofing.com/</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>South Florida</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>office@stat-roofing.com</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>(561) 840-0504</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>West Palm Beach FL</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>roof replacement West Palm Beach FL</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-12 00:11 UTC (cycle 170)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-12.xlsx
+++ b/output/leads_2026-10-12.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -623,6 +623,66 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg HVAC – Furnace &amp; Heat Pump Install, AC Repair &amp; Mini-Split Service | </t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>heisenbergwa.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://heisenbergwa.com/heat-pump-installation-vancouver-wa/</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Maintenance Plans</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>heisenberghvac@gmail.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>971-294-1215</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Vancouver WA</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>100</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>heat pump installation Vancouver WA</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-12 00:14 UTC (cycle 172)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-12.xlsx
+++ b/output/leads_2026-10-12.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -683,6 +683,62 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>HVAC Contractor Precision Mechanical Solutions</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>precisionmechanicalsolutions.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://www.precisionmechanicalsolutions.com/</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>dispatch@pmsihvac.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>(559) 347-9500</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Fresno CA</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>100</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>HVAC contractor Fresno CA</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-12 05:25 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-12.xlsx
+++ b/output/leads_2026-10-12.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -704,7 +704,6 @@
           <t>https://www.precisionmechanicalsolutions.com/</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>dispatch@pmsihvac.com</t>
@@ -734,6 +733,66 @@
         </is>
       </c>
       <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Plumber Honolulu Hawaii</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>plumbershonoluluhawaii.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://www.plumbershonoluluhawaii.com/</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Plumber Honolulu</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>info@plumbershonoluluhawaii.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>844-833-1546</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Honolulu HI</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>100</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>emergency plumber Honolulu HI</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
         <is>
           <t>2026-10-12</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-12 05:27 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-12.xlsx
+++ b/output/leads_2026-10-12.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -798,6 +798,66 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Emergency Plumber in Renton, WA | Plumbing Experts Renton</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>plumbingexpertsrenton.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://plumbingexpertsrenton.com/</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Plumbing Experts</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>contact@plumbingexpertsrenton.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>(425) 380-0167</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Renton WA</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>90</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>emergency plumber Renton WA</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-12 05:30 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-12.xlsx
+++ b/output/leads_2026-10-12.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -858,6 +858,66 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Roof Replacement in Cape Coral, FL | Blue Dog Roofing &amp; Construction</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>bluedogrc.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://bluedogrc.com/roofing-cape-coral-fl.html</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Estimate For</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>admin@bluedogrc.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>(239) 888-1008</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Cape Coral FL</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>100</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>roof replacement Cape Coral FL</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-12 17:46 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-12.xlsx
+++ b/output/leads_2026-10-12.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -918,6 +918,66 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Benjamin Franklin Plumbing</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>benjaminfranklinplumbingfortworth.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://benjaminfranklinplumbingfortworth.com/sewer-drains/trenchless-sewer-repair/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Slab Leak</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>service@benfranklinarlington.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>817-983-7876</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Fort Worth TX</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>100</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>sewer repair Fort Worth TX</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-12 17:52 UTC (cycle 11)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-12.xlsx
+++ b/output/leads_2026-10-12.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -978,6 +978,66 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Zana Roofing &amp; Construction</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>zanaroofing.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://zanaroofing.com/</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Northeast Ohio</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>contact@zanaroofing.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>(831) 666-1600</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Youngstown OH</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>100</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>roofing contractor Youngstown OH</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-12 20:06 UTC (cycle 66)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-12.xlsx
+++ b/output/leads_2026-10-12.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1038,6 +1038,58 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>JC Sewer &amp; Drain Plumbing Inc | Stockton's Neighborhood Plumber</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>jcseweranddrain.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://jcseweranddrain.com/sewer-line-repair</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>jcseweranddrain@gmail.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Stockton CA</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>72</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>sewer repair Stockton CA</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>